<commit_message>
Name and Group swap on reformatted header
</commit_message>
<xml_diff>
--- a/metab_neg_reformatted.xlsx
+++ b/metab_neg_reformatted.xlsx
@@ -487,12 +487,12 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
           <t>Group</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">

</xml_diff>